<commit_message>
Implement basic functionality for beverage mixer including HX711 weight measurement and GPIO setup for pumps and sensors. Add initial test script for basic output.
</commit_message>
<xml_diff>
--- a/Anschlussplan.xlsx
+++ b/Anschlussplan.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://voithprod-my.sharepoint.com/personal/laurin_oberlader_voith_com/Documents/Studium/Fächer/Informatik/Informatik 2/Projektarbeit/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="22" documentId="8_{69C211D4-98CC-4043-94C0-45C4F311E0A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EB1CEF21-1676-4645-A9F9-1E3CFD418FC4}"/>
+  <xr:revisionPtr revIDLastSave="46" documentId="8_{69C211D4-98CC-4043-94C0-45C4F311E0A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4AD853A7-8A7A-4A95-BA44-E798FC01F4A6}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{30C6F8F9-7A31-455B-BCE7-BC90DC021967}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="13056" xr2:uid="{30C6F8F9-7A31-455B-BCE7-BC90DC021967}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="23">
   <si>
     <t>Anschlussplan Raspberry Pi Pico</t>
   </si>
@@ -56,21 +56,6 @@
     <t>DI</t>
   </si>
   <si>
-    <t>Sensor 1</t>
-  </si>
-  <si>
-    <t>Sensor 2</t>
-  </si>
-  <si>
-    <t>Sensor 3</t>
-  </si>
-  <si>
-    <t>Sensor 4</t>
-  </si>
-  <si>
-    <t>Sensor 5</t>
-  </si>
-  <si>
     <t>Pumpe 1</t>
   </si>
   <si>
@@ -83,9 +68,6 @@
     <t>Pumpe 4</t>
   </si>
   <si>
-    <t>Pumpe 5</t>
-  </si>
-  <si>
     <t>GND</t>
   </si>
   <si>
@@ -99,6 +81,30 @@
   </si>
   <si>
     <t>VSYS</t>
+  </si>
+  <si>
+    <t>sck</t>
+  </si>
+  <si>
+    <t>Puls</t>
+  </si>
+  <si>
+    <t>Wägezelle 1</t>
+  </si>
+  <si>
+    <t>Wägezelle 2</t>
+  </si>
+  <si>
+    <t>Wägezelle 3</t>
+  </si>
+  <si>
+    <t>Wägezelle 4</t>
+  </si>
+  <si>
+    <t>0V Pumpen</t>
+  </si>
+  <si>
+    <t>0V Sensoren</t>
   </si>
 </sst>
 </file>
@@ -147,7 +153,17 @@
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="3">
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -160,14 +176,18 @@
 </styleSheet>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{0039DDD8-9F60-4BB0-B93F-512C3E588B76}" name="Tabelle3" displayName="Tabelle3" ref="A3:D15" totalsRowShown="0">
   <autoFilter ref="A3:D15" xr:uid="{0039DDD8-9F60-4BB0-B93F-512C3E588B76}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{31C7B293-9963-44A5-B65A-F9AC45C5E892}" name="Anschluss"/>
-    <tableColumn id="2" xr3:uid="{EA265DF8-BE97-4EC4-8BAE-8037526D1128}" name="GPIO"/>
-    <tableColumn id="3" xr3:uid="{4271BE4A-7DF1-4A73-8000-EF784356ED0B}" name="Pin Nr."/>
-    <tableColumn id="4" xr3:uid="{A24BB3AD-865C-4A3C-B42E-C03A0C5F291D}" name="Funktion"/>
+    <tableColumn id="2" xr3:uid="{EA265DF8-BE97-4EC4-8BAE-8037526D1128}" name="GPIO" dataDxfId="0"/>
+    <tableColumn id="3" xr3:uid="{4271BE4A-7DF1-4A73-8000-EF784356ED0B}" name="Pin Nr." dataDxfId="1"/>
+    <tableColumn id="4" xr3:uid="{A24BB3AD-865C-4A3C-B42E-C03A0C5F291D}" name="Funktion" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -492,6 +512,12 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{29536A51-6EC8-44E5-8273-1946B829D5F9}">
   <dimension ref="A1:D15"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="13.69921875" customWidth="1"/>
+    <col min="2" max="2" width="7.3984375" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.69921875" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.19921875" style="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
@@ -502,182 +528,182 @@
       <c r="A3" t="s">
         <v>1</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" s="1" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>6</v>
-      </c>
-      <c r="B4">
+        <v>15</v>
+      </c>
+      <c r="B4" s="1">
         <v>0</v>
       </c>
-      <c r="C4">
+      <c r="C4" s="1">
         <v>1</v>
       </c>
-      <c r="D4" t="s">
-        <v>5</v>
+      <c r="D4" s="1" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>7</v>
-      </c>
-      <c r="B5">
+        <v>17</v>
+      </c>
+      <c r="B5" s="1">
         <v>1</v>
       </c>
-      <c r="C5">
+      <c r="C5" s="1">
         <v>2</v>
       </c>
-      <c r="D5" t="s">
+      <c r="D5" s="1" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>8</v>
-      </c>
-      <c r="B6">
+        <v>18</v>
+      </c>
+      <c r="B6" s="1">
         <v>2</v>
       </c>
-      <c r="C6">
+      <c r="C6" s="1">
         <v>4</v>
       </c>
-      <c r="D6" t="s">
+      <c r="D6" s="1" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>9</v>
-      </c>
-      <c r="B7">
+        <v>19</v>
+      </c>
+      <c r="B7" s="1">
         <v>3</v>
       </c>
-      <c r="C7">
+      <c r="C7" s="1">
         <v>5</v>
       </c>
-      <c r="D7" t="s">
+      <c r="D7" s="1" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>10</v>
-      </c>
-      <c r="B8">
+        <v>20</v>
+      </c>
+      <c r="B8" s="1">
         <v>4</v>
       </c>
-      <c r="C8">
+      <c r="C8" s="1">
         <v>6</v>
       </c>
-      <c r="D8" t="s">
+      <c r="D8" s="1" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>6</v>
+      </c>
+      <c r="B9" s="1">
+        <v>16</v>
+      </c>
+      <c r="C9" s="1">
+        <v>14</v>
+      </c>
+      <c r="D9" s="1" t="s">
         <v>11</v>
-      </c>
-      <c r="B9">
-        <v>22</v>
-      </c>
-      <c r="C9">
-        <v>14</v>
-      </c>
-      <c r="D9" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>12</v>
-      </c>
-      <c r="B10">
-        <v>21</v>
-      </c>
-      <c r="C10">
+        <v>7</v>
+      </c>
+      <c r="B10" s="1">
+        <v>17</v>
+      </c>
+      <c r="C10" s="1">
         <v>16</v>
       </c>
-      <c r="D10" t="s">
-        <v>17</v>
+      <c r="D10" s="1" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>13</v>
-      </c>
-      <c r="B11">
+        <v>8</v>
+      </c>
+      <c r="B11" s="1">
         <v>20</v>
       </c>
-      <c r="C11">
+      <c r="C11" s="1">
         <v>18</v>
       </c>
-      <c r="D11" t="s">
-        <v>17</v>
+      <c r="D11" s="1" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>14</v>
-      </c>
-      <c r="B12">
-        <v>19</v>
-      </c>
-      <c r="C12">
+        <v>9</v>
+      </c>
+      <c r="B12" s="1">
+        <v>21</v>
+      </c>
+      <c r="C12" s="1">
         <v>20</v>
       </c>
-      <c r="D12" t="s">
-        <v>17</v>
+      <c r="D12" s="1" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>15</v>
-      </c>
-      <c r="B13">
-        <v>18</v>
-      </c>
-      <c r="C13">
-        <v>22</v>
-      </c>
-      <c r="D13" t="s">
-        <v>17</v>
+        <v>12</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C13" s="1">
+        <v>39</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>18</v>
-      </c>
-      <c r="B14" t="s">
-        <v>20</v>
-      </c>
-      <c r="C14">
-        <v>39</v>
-      </c>
-      <c r="D14" t="s">
-        <v>18</v>
+        <v>13</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C14" s="1">
+        <v>3</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>22</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>19</v>
-      </c>
-      <c r="B15" t="s">
-        <v>16</v>
-      </c>
-      <c r="C15">
-        <v>3</v>
-      </c>
-      <c r="D15" t="s">
-        <v>19</v>
+        <v>13</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C15" s="1">
+        <v>23</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>